<commit_message>
docs(travel): BẬT visa nhóm Quảng Châu (D11=1) + nhãn Canton Fair 2 người tách riêng
- QC cần visa TQ (đi Canton Fair + tour) → ThamSo D11=1 cả 3 option, recalc:
  TỔNG đoàn A 314,53tr · B 314,01tr · C 328,95tr (QC/người +~2,49tr)
- Vé bay + KS Canton Fair là cho 2 người, ĐỂ RIÊNG khỏi ngân sách tour (Sếp chốt)
- Cập nhật bảng 4.1/4.2, điểm chốt #5 ✅, ghi chú so v3

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/travel/tour-china-2026-10-budget-optB.xlsx
+++ b/docs/travel/tour-china-2026-10-budget-optB.xlsx
@@ -738,7 +738,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -1896,19 +1896,19 @@
       </c>
       <c r="C6" s="18">
         <f>ChiPhi_QC!$D$23</f>
-        <v>31680075</v>
+        <v>33937675</v>
       </c>
       <c r="D6" s="18">
         <f>ChiPhi_QC!$D$25</f>
-        <v>34848082.5</v>
+        <v>37331442.5</v>
       </c>
       <c r="E6" s="18">
         <f>ChiPhi_QC!$E$23</f>
-        <v>63360150</v>
+        <v>67875350</v>
       </c>
       <c r="F6" s="18">
         <f>ChiPhi_QC!$E$25</f>
-        <v>69696165</v>
+        <v>74662885</v>
       </c>
     </row>
     <row r="7">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="F7" s="20">
         <f>SUM(F4:F6)</f>
-        <v>309041205</v>
+        <v>314007925</v>
       </c>
     </row>
     <row r="9">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="C5" s="40">
         <f>TODAY()</f>
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B4" s="17">
         <f>ThamSo!$D$11</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -5491,7 +5491,7 @@
       </c>
       <c r="B7" s="41">
         <f>$B$4</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" s="29">
         <f>ThamSo!$B$59*ThamSo!$B$5+ThamSo!$B$60</f>
@@ -5499,11 +5499,11 @@
       </c>
       <c r="D7" s="29">
         <f>B7*C7</f>
-        <v>0</v>
+        <v>2257600</v>
       </c>
       <c r="E7" s="29">
         <f>D7*$B$2</f>
-        <v>0</v>
+        <v>4515200</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -5935,7 +5935,7 @@
       </c>
       <c r="E23" s="31">
         <f>SUM(E7:E22)</f>
-        <v>63360150</v>
+        <v>67875350</v>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
@@ -5951,11 +5951,11 @@
       </c>
       <c r="D24" s="29">
         <f>D23*ThamSo!$B$6</f>
-        <v>3168007.5</v>
+        <v>3393767.5</v>
       </c>
       <c r="E24" s="29">
         <f>E23*ThamSo!$B$6</f>
-        <v>6336015</v>
+        <v>6787535</v>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
@@ -5971,11 +5971,11 @@
       </c>
       <c r="D25" s="20">
         <f>D23+D24</f>
-        <v>34848082.5</v>
+        <v>37331442.5</v>
       </c>
       <c r="E25" s="20">
         <f>E23+E24</f>
-        <v>69696165</v>
+        <v>74662885</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(travel): chặng VỀ bay đêm (Air China + VJ3949 04/11) + bay HGH→BK thay tàu + lịch chi tiết cả 3 option
- HN về: Air China PEK→HAN 00:10→03:15 đêm 04/11 = 3.094.000đ (rẻ hơn Xiamen, bay đêm → chơi trọn ngày cuối)
- SGN+QC về: VJ3949 PKX→SGN 01:05→05:10 đêm 04/11 = 3.753.000đ (Option C dùng giá 05/11)
- Hàng Châu→Bắc Kinh: ĐỔI tàu 650 CNY sang BAY ~520 CNY (rẻ & nhanh hơn)
- Viết lịch giờ-by-giờ đầy đủ cho cả 3 option (A/B/C)
- Recalc: TỔNG đoàn A 307,22tr · B 306,70tr · C 324,58tr; bảng 4 + điểm chốt cập nhật

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/travel/tour-china-2026-10-budget-optB.xlsx
+++ b/docs/travel/tour-china-2026-10-budget-optB.xlsx
@@ -995,21 +995,21 @@
         </is>
       </c>
       <c r="B26" s="33" t="n">
-        <v>152</v>
+        <v>3094000</v>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>VND</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>XiamenAir PKX 15:10 → HAN 17:55 (bay thẳng ban NGÀY; đêm 03→04/11 KHÔNG có VietJet thẳng)</t>
+          <t>Air China PEK 00:10 → HAN 03:15 (bay thẳng ĐÊM, từ Bắc Kinh Thủ Đô PEK)</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Trip.com+Google 22/09: nonstop chỉ Xiamen ban ngày $152; VERIFY app Vietjet lúc book</t>
+          <t>Ảnh Sếp 23/09: 3.105.000đ; rẻ hơn Xiamen + bay đêm, giữ ngày cuối</t>
         </is>
       </c>
     </row>
@@ -1020,11 +1020,11 @@
         </is>
       </c>
       <c r="B27" s="33" t="n">
-        <v>148</v>
+        <v>3753000</v>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>VND</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Trip.com 22/09: VJ3949 $148 (exclusive fare); đặt thẳng Vietjet.com có thể ~$110</t>
+          <t>Ảnh Sếp 23/09: VJ3949 4.126.000đ (từ PKX Đại Hưng)</t>
         </is>
       </c>
     </row>
@@ -1091,11 +1091,11 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Tàu Hangzhou East → Beijing South hạng 2</t>
+          <t>Bay Hàng Châu → Bắc Kinh (~2h15)</t>
         </is>
       </c>
       <c r="B30" s="33" t="n">
-        <v>650</v>
+        <v>520</v>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
@@ -1104,12 +1104,12 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Tàu G ~4,5–5h, mở bán 15 ngày trước</t>
+          <t>Bay HGH → Bắc Kinh (China Eastern ~2h15), THAY tàu; + transfer sân bay ~1h</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>travelchinaguide 2026: 605–749 CNY</t>
+          <t>Trip.com 23/09: bay thẳng 480–560 CNY, rẻ &amp; nhanh hơn tàu 650</t>
         </is>
       </c>
     </row>
@@ -1842,19 +1842,19 @@
       </c>
       <c r="C4" s="18">
         <f>ChiPhi_HN!$D$23</f>
-        <v>37679740</v>
+        <v>36276320</v>
       </c>
       <c r="D4" s="18">
         <f>ChiPhi_HN!$D$25</f>
-        <v>41447714</v>
+        <v>39903952</v>
       </c>
       <c r="E4" s="18">
         <f>ChiPhi_HN!$E$23</f>
-        <v>75359480</v>
+        <v>72552640</v>
       </c>
       <c r="F4" s="18">
         <f>ChiPhi_HN!$E$25</f>
-        <v>82895428</v>
+        <v>79807904</v>
       </c>
     </row>
     <row r="5">
@@ -1869,19 +1869,19 @@
       </c>
       <c r="C5" s="18">
         <f>ChiPhi_SGN!$D$23</f>
-        <v>35556730</v>
+        <v>34917150</v>
       </c>
       <c r="D5" s="18">
         <f>ChiPhi_SGN!$D$25</f>
-        <v>39112403</v>
+        <v>38408865</v>
       </c>
       <c r="E5" s="18">
         <f>ChiPhi_SGN!$E$23</f>
-        <v>142226920</v>
+        <v>139668600</v>
       </c>
       <c r="F5" s="18">
         <f>ChiPhi_SGN!$E$25</f>
-        <v>156449612</v>
+        <v>153635460</v>
       </c>
     </row>
     <row r="6">
@@ -1896,19 +1896,19 @@
       </c>
       <c r="C6" s="18">
         <f>ChiPhi_QC!$D$23</f>
-        <v>33937675</v>
+        <v>33298095</v>
       </c>
       <c r="D6" s="18">
         <f>ChiPhi_QC!$D$25</f>
-        <v>37331442.5</v>
+        <v>36627904.5</v>
       </c>
       <c r="E6" s="18">
         <f>ChiPhi_QC!$E$23</f>
-        <v>67875350</v>
+        <v>66596190</v>
       </c>
       <c r="F6" s="18">
         <f>ChiPhi_QC!$E$25</f>
-        <v>74662885</v>
+        <v>73255809</v>
       </c>
     </row>
     <row r="7">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="F7" s="20">
         <f>SUM(F4:F6)</f>
-        <v>314007925</v>
+        <v>306699173</v>
       </c>
     </row>
     <row r="9">
@@ -4371,15 +4371,15 @@
       </c>
       <c r="C9" s="29">
         <f>IF(ThamSo!$C$26="CNY",ThamSo!$B$26*ThamSo!$B$4,IF(ThamSo!$C$26="USD",ThamSo!$B$26*ThamSo!$B$5,ThamSo!$B$26))</f>
-        <v>3983920</v>
+        <v>3094000</v>
       </c>
       <c r="D9" s="29">
         <f>B9*C9</f>
-        <v>3983920</v>
+        <v>3094000</v>
       </c>
       <c r="E9" s="29">
         <f>D9*$B$2</f>
-        <v>7967840</v>
+        <v>6188000</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -4452,15 +4452,15 @@
       </c>
       <c r="C12" s="29">
         <f>IF(ThamSo!$C$30="CNY",ThamSo!$B$30*ThamSo!$B$4,IF(ThamSo!$C$30="USD",ThamSo!$B$30*ThamSo!$B$5,ThamSo!$B$30))</f>
-        <v>2567500</v>
+        <v>2054000</v>
       </c>
       <c r="D12" s="29">
         <f>B12*C12</f>
-        <v>2567500</v>
+        <v>2054000</v>
       </c>
       <c r="E12" s="29">
         <f>D12*$B$2</f>
-        <v>5135000</v>
+        <v>4108000</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -4757,7 +4757,7 @@
       </c>
       <c r="E23" s="31">
         <f>SUM(E7:E22)</f>
-        <v>75359480</v>
+        <v>72552640</v>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
@@ -4773,11 +4773,11 @@
       </c>
       <c r="D24" s="29">
         <f>D23*ThamSo!$B$6</f>
-        <v>3767974</v>
+        <v>3627632</v>
       </c>
       <c r="E24" s="29">
         <f>E23*ThamSo!$B$6</f>
-        <v>7535948</v>
+        <v>7255264</v>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
@@ -4793,11 +4793,11 @@
       </c>
       <c r="D25" s="20">
         <f>D23+D24</f>
-        <v>41447714</v>
+        <v>39903952</v>
       </c>
       <c r="E25" s="20">
         <f>E23+E24</f>
-        <v>82895428</v>
+        <v>79807904</v>
       </c>
     </row>
   </sheetData>
@@ -4960,15 +4960,15 @@
       </c>
       <c r="C9" s="29">
         <f>IF(ThamSo!$C$27="CNY",ThamSo!$B$27*ThamSo!$B$4,IF(ThamSo!$C$27="USD",ThamSo!$B$27*ThamSo!$B$5,ThamSo!$B$27))</f>
-        <v>3879080</v>
+        <v>3753000</v>
       </c>
       <c r="D9" s="29">
         <f>B9*C9</f>
-        <v>3879080</v>
+        <v>3753000</v>
       </c>
       <c r="E9" s="29">
         <f>D9*$B$2</f>
-        <v>15516320</v>
+        <v>15012000</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -5041,15 +5041,15 @@
       </c>
       <c r="C12" s="29">
         <f>IF(ThamSo!$C$30="CNY",ThamSo!$B$30*ThamSo!$B$4,IF(ThamSo!$C$30="USD",ThamSo!$B$30*ThamSo!$B$5,ThamSo!$B$30))</f>
-        <v>2567500</v>
+        <v>2054000</v>
       </c>
       <c r="D12" s="29">
         <f>B12*C12</f>
-        <v>2567500</v>
+        <v>2054000</v>
       </c>
       <c r="E12" s="29">
         <f>D12*$B$2</f>
-        <v>10270000</v>
+        <v>8216000</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="E23" s="31">
         <f>SUM(E7:E22)</f>
-        <v>142226920</v>
+        <v>139668600</v>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
@@ -5362,11 +5362,11 @@
       </c>
       <c r="D24" s="29">
         <f>D23*ThamSo!$B$6</f>
-        <v>3555673</v>
+        <v>3491715</v>
       </c>
       <c r="E24" s="29">
         <f>E23*ThamSo!$B$6</f>
-        <v>14222692</v>
+        <v>13966860</v>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
@@ -5382,11 +5382,11 @@
       </c>
       <c r="D25" s="20">
         <f>D23+D24</f>
-        <v>39112403</v>
+        <v>38408865</v>
       </c>
       <c r="E25" s="20">
         <f>E23+E24</f>
-        <v>156449612</v>
+        <v>153635460</v>
       </c>
     </row>
   </sheetData>
@@ -5549,15 +5549,15 @@
       </c>
       <c r="C9" s="29">
         <f>IF(ThamSo!$C$27="CNY",ThamSo!$B$27*ThamSo!$B$4,IF(ThamSo!$C$27="USD",ThamSo!$B$27*ThamSo!$B$5,ThamSo!$B$27))</f>
-        <v>3879080</v>
+        <v>3753000</v>
       </c>
       <c r="D9" s="29">
         <f>B9*C9</f>
-        <v>3879080</v>
+        <v>3753000</v>
       </c>
       <c r="E9" s="29">
         <f>D9*$B$2</f>
-        <v>7758160</v>
+        <v>7506000</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -5630,15 +5630,15 @@
       </c>
       <c r="C12" s="29">
         <f>IF(ThamSo!$C$30="CNY",ThamSo!$B$30*ThamSo!$B$4,IF(ThamSo!$C$30="USD",ThamSo!$B$30*ThamSo!$B$5,ThamSo!$B$30))</f>
-        <v>2567500</v>
+        <v>2054000</v>
       </c>
       <c r="D12" s="29">
         <f>B12*C12</f>
-        <v>2567500</v>
+        <v>2054000</v>
       </c>
       <c r="E12" s="29">
         <f>D12*$B$2</f>
-        <v>5135000</v>
+        <v>4108000</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -5935,7 +5935,7 @@
       </c>
       <c r="E23" s="31">
         <f>SUM(E7:E22)</f>
-        <v>67875350</v>
+        <v>66596190</v>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
@@ -5951,11 +5951,11 @@
       </c>
       <c r="D24" s="29">
         <f>D23*ThamSo!$B$6</f>
-        <v>3393767.5</v>
+        <v>3329809.5</v>
       </c>
       <c r="E24" s="29">
         <f>E23*ThamSo!$B$6</f>
-        <v>6787535</v>
+        <v>6659619</v>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
@@ -5971,11 +5971,11 @@
       </c>
       <c r="D25" s="20">
         <f>D23+D24</f>
-        <v>37331442.5</v>
+        <v>36627904.5</v>
       </c>
       <c r="E25" s="20">
         <f>E23+E24</f>
-        <v>74662885</v>
+        <v>73255809</v>
       </c>
     </row>
   </sheetData>

</xml_diff>